<commit_message>
Actualizar checklist de fotos con las imágenes del nuevo slider
Sustituye las 4 filas de las antiguas imágenes de colección
(coleccion-signature/nupcial/esmeraldas/zafiros.jpg, ya no usadas en
index.old.html) por las 8 imágenes del nuevo slider "Piezas que
enamoran": home-slider-anillos/pendientes/collares/pulseras.jpg y
home-destacado-1 a 4.jpg, con medidas, descripción y prompt sugerido
para cada una.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G17"/>
+  <dimension ref="A2:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -685,7 +685,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>coleccion-signature.jpg</t>
+          <t>home-slider-anillos.jpg</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -695,23 +695,23 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Colección Signature</t>
+          <t>Piezas que enamoran — Anillos (modelo)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>800×800 px
-≤150 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Pieza icónica de la colección Signature: anillo o collar en oro con piedra preciosa. Cuadrada, centrada.</t>
+          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Iconic gold ring with a brilliant cut diamond on white marble surface, luxury jewelry product photography, top-down view, perfect symmetry, soft shadows, 8K, minimal</t>
+          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>coleccion-nupcial.jpg</t>
+          <t>home-slider-pendientes.jpg</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -731,23 +731,23 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Colección Nupcial</t>
+          <t>Piezas que enamoran — Pendientes (estudio)</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>800×800 px
-≤150 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Alianzas de boda o anillo de compromiso. Ambiente romántico, flores blancas o seda.</t>
+          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Elegant wedding rings and engagement ring with diamond on white silk fabric with white rose petals, romantic luxury jewelry photography, soft bokeh, pastel tones, 8K</t>
+          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>coleccion-esmeraldas.jpg</t>
+          <t>home-slider-collares.jpg</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -767,23 +767,23 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Colección Esmeraldas</t>
+          <t>Piezas que enamoran — Collares (estudio)</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>800×800 px
-≤150 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Joya protagonizada por esmeraldas: pendientes o anillo. Fondo que resalte el verde.</t>
+          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Luxury emerald and gold earrings on dark green velvet background, dramatic lighting, vivid green gemstones, fine jewelry photography, sharp and detailed, editorial style, 8K</t>
+          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>coleccion-zafiros.jpg</t>
+          <t>home-slider-pulseras.jpg</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -803,23 +803,23 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Colección Zafiros</t>
+          <t>Piezas que enamoran — Pulseras (modelo)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>800×800 px
-≤150 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Pieza con zafiros azules. Fondo oscuro o azul profundo para resaltar el color de la gema.</t>
+          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Sapphire and white gold bracelet on deep navy velvet, vibrant blue gemstones, luxury jewelry editorial photography, dramatic studio light, 8K, ultra detailed</t>
+          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
     </row>
@@ -829,33 +829,33 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>proceso-boceto.jpg</t>
+          <t>home-destacado-1.jpg</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Paso 1 — Boceto</t>
+          <t>Piezas destacadas — pieza 1</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -865,33 +865,33 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>proceso-materiales.jpg</t>
+          <t>home-destacado-2.jpg</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Paso 2 — Materiales</t>
+          <t>Piezas destacadas — pieza 2</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -901,33 +901,33 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>proceso-artesania.jpg</t>
+          <t>home-destacado-3.jpg</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Paso 3 — Artesanía</t>
+          <t>Piezas destacadas — pieza 3</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -937,38 +937,183 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>proceso-entrega.jpg</t>
+          <t>home-destacado-4.jpg</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Piezas destacadas — pieza 4</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>800×1000 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>proceso-boceto.jpg</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Paso 4 — Entrega</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Paso 1 — Boceto</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>proceso-materiales.jpg</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Paso 2 — Materiales</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>proceso-artesania.jpg</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Paso 3 — Artesanía</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="70" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>proceso-entrega.jpg</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Paso 4 — Entrega</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Joya terminada en estuche o caja de regalo de lujo. Momento de entrega o presentación.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen</t>
         </is>
@@ -976,8 +1121,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A17:G17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar checklist de fotos con las imágenes del nuevo slider (#4)
Sustituye las 4 filas de las antiguas imágenes de colección
(coleccion-signature/nupcial/esmeraldas/zafiros.jpg, ya no usadas en
index.old.html) por las 8 imágenes del nuevo slider "Piezas que
enamoran": home-slider-anillos/pendientes/collares/pulseras.jpg y
home-destacado-1 a 4.jpg, con medidas, descripción y prompt sugerido
para cada una.


Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G17"/>
+  <dimension ref="A2:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -685,7 +685,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>coleccion-signature.jpg</t>
+          <t>home-slider-anillos.jpg</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -695,23 +695,23 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Colección Signature</t>
+          <t>Piezas que enamoran — Anillos (modelo)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>800×800 px
-≤150 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Pieza icónica de la colección Signature: anillo o collar en oro con piedra preciosa. Cuadrada, centrada.</t>
+          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Iconic gold ring with a brilliant cut diamond on white marble surface, luxury jewelry product photography, top-down view, perfect symmetry, soft shadows, 8K, minimal</t>
+          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>coleccion-nupcial.jpg</t>
+          <t>home-slider-pendientes.jpg</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -731,23 +731,23 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Colección Nupcial</t>
+          <t>Piezas que enamoran — Pendientes (estudio)</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>800×800 px
-≤150 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Alianzas de boda o anillo de compromiso. Ambiente romántico, flores blancas o seda.</t>
+          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Elegant wedding rings and engagement ring with diamond on white silk fabric with white rose petals, romantic luxury jewelry photography, soft bokeh, pastel tones, 8K</t>
+          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>coleccion-esmeraldas.jpg</t>
+          <t>home-slider-collares.jpg</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -767,23 +767,23 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Colección Esmeraldas</t>
+          <t>Piezas que enamoran — Collares (estudio)</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>800×800 px
-≤150 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Joya protagonizada por esmeraldas: pendientes o anillo. Fondo que resalte el verde.</t>
+          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Luxury emerald and gold earrings on dark green velvet background, dramatic lighting, vivid green gemstones, fine jewelry photography, sharp and detailed, editorial style, 8K</t>
+          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>coleccion-zafiros.jpg</t>
+          <t>home-slider-pulseras.jpg</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -803,23 +803,23 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Colección Zafiros</t>
+          <t>Piezas que enamoran — Pulseras (modelo)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>800×800 px
-≤150 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Pieza con zafiros azules. Fondo oscuro o azul profundo para resaltar el color de la gema.</t>
+          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Sapphire and white gold bracelet on deep navy velvet, vibrant blue gemstones, luxury jewelry editorial photography, dramatic studio light, 8K, ultra detailed</t>
+          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
     </row>
@@ -829,33 +829,33 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>proceso-boceto.jpg</t>
+          <t>home-destacado-1.jpg</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Paso 1 — Boceto</t>
+          <t>Piezas destacadas — pieza 1</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -865,33 +865,33 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>proceso-materiales.jpg</t>
+          <t>home-destacado-2.jpg</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Paso 2 — Materiales</t>
+          <t>Piezas destacadas — pieza 2</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -901,33 +901,33 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>proceso-artesania.jpg</t>
+          <t>home-destacado-3.jpg</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Paso 3 — Artesanía</t>
+          <t>Piezas destacadas — pieza 3</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -937,38 +937,183 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>proceso-entrega.jpg</t>
+          <t>home-destacado-4.jpg</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Piezas destacadas — pieza 4</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>800×1000 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>proceso-boceto.jpg</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Paso 4 — Entrega</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Paso 1 — Boceto</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>proceso-materiales.jpg</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Paso 2 — Materiales</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>proceso-artesania.jpg</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Paso 3 — Artesanía</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="70" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>proceso-entrega.jpg</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Paso 4 — Entrega</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Joya terminada en estuche o caja de regalo de lujo. Momento de entrega o presentación.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen</t>
         </is>
@@ -976,8 +1121,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A17:G17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mover las fotos del slider de home a images/home/
Crea la carpeta images/home/ para las 8 imágenes del slider "Piezas
que enamoran" (home-slider-*.jpg, home-destacado-*.jpg) en lugar de
dejarlas sueltas en la raíz del repo, junto al resto de HTML. Se
actualizan las rutas en index.old.html y en el checklist de fotos
para que apunten a la nueva carpeta.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -517,7 +517,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -685,7 +685,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>home-slider-anillos.jpg</t>
+          <t>images/home/home-slider-anillos.jpg</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>home-slider-pendientes.jpg</t>
+          <t>images/home/home-slider-pendientes.jpg</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>home-slider-collares.jpg</t>
+          <t>images/home/home-slider-collares.jpg</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>home-slider-pulseras.jpg</t>
+          <t>images/home/home-slider-pulseras.jpg</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>home-destacado-1.jpg</t>
+          <t>images/home/home-destacado-1.jpg</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>home-destacado-2.jpg</t>
+          <t>images/home/home-destacado-2.jpg</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>home-destacado-3.jpg</t>
+          <t>images/home/home-destacado-3.jpg</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>home-destacado-4.jpg</t>
+          <t>images/home/home-destacado-4.jpg</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1111,7 +1111,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mover las fotos del slider de home a images/home/ (#5)
Crea la carpeta images/home/ para las 8 imágenes del slider "Piezas
que enamoran" (home-slider-*.jpg, home-destacado-*.jpg) en lugar de
dejarlas sueltas en la raíz del repo, junto al resto de HTML. Se
actualizan las rutas en index.old.html y en el checklist de fotos
para que apunten a la nueva carpeta.


Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -517,7 +517,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -685,7 +685,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>home-slider-anillos.jpg</t>
+          <t>images/home/home-slider-anillos.jpg</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>home-slider-pendientes.jpg</t>
+          <t>images/home/home-slider-pendientes.jpg</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>home-slider-collares.jpg</t>
+          <t>images/home/home-slider-collares.jpg</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>home-slider-pulseras.jpg</t>
+          <t>images/home/home-slider-pulseras.jpg</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>home-destacado-1.jpg</t>
+          <t>images/home/home-destacado-1.jpg</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>home-destacado-2.jpg</t>
+          <t>images/home/home-destacado-2.jpg</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>home-destacado-3.jpg</t>
+          <t>images/home/home-destacado-3.jpg</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>home-destacado-4.jpg</t>
+          <t>images/home/home-destacado-4.jpg</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1111,7 +1111,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Añadir 2ª foto en hover a las 3 imágenes del hero
Cada una de las 3 fotos del hero principal ahora muestra una segunda
imagen con un fundido suave al pasar el ratón por encima, sin
necesidad de hacer clic (foto-principal-modelo.jpg, foto-hero-2-modelo.jpg,
foto-hero-3-modelo.jpg). Pensado para alternar la foto de estudio con
la pieza puesta en modelo. Se actualiza el checklist de fotos con las
3 nuevas filas y sus prompts sugeridos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G21"/>
+  <dimension ref="A2:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -613,7 +613,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>foto-hero-2.jpg</t>
+          <t>foto-principal-modelo.jpg</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Hero slider 2</t>
+          <t>Hero principal — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -634,12 +634,12 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Atelier o taller joyero: mesa de trabajo con herramientas artesanales, bocetos y materiales.</t>
+          <t>Se muestra al pasar el ratón sobre la foto principal, sin hacer clic. Misma joya puesta en modelo, para contrastar con la foto de estudio.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Luxury jewelry atelier workbench with golden tools, gemstones, sketches and magnifying glass, warm soft light, shallow depth of field, artisan craftsmanship, elegant editorial photography, 8K</t>
+          <t>The same exquisite gold diamond ring worn on an elegant female hand, editorial luxury jewelry campaign photography, soft natural light, neutral cream background, high-end style, ultra sharp, 8K</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>foto-hero-3.jpg</t>
+          <t>foto-hero-2.jpg</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Hero slider 3</t>
+          <t>Hero slider 2</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -670,12 +670,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Collar o pendientes en expositor de terciopelo oscuro. Iluminación de joyería de lujo.</t>
+          <t>Atelier o taller joyero: mesa de trabajo con herramientas artesanales, bocetos y materiales.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Fine jewelry necklace with emeralds displayed on dark velvet, dramatic studio lighting, luxury brand photography, high contrast, ultra sharp details, elegant and minimal, 8K</t>
+          <t>Luxury jewelry atelier workbench with golden tools, gemstones, sketches and magnifying glass, warm soft light, shallow depth of field, artisan craftsmanship, elegant editorial photography, 8K</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>images/home/home-slider-anillos.jpg</t>
+          <t>foto-hero-2-modelo.jpg</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -695,23 +695,23 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Anillos (modelo)</t>
+          <t>Hero slider 2 — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>1200×1500 px
-≤400 KB</t>
+          <t>1920×1080 px
+≤300 KB</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
+          <t>Se muestra al pasar el ratón sobre la foto 2, sin hacer clic. El anillo protagonista puesto en modelo, en vez de la vista del taller.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
+          <t>Close-up of a woman's hand wearing an elegant gold ring, editorial luxury jewelry campaign photography, warm soft light, shallow depth of field, elegant style, 8K</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>images/home/home-slider-pendientes.jpg</t>
+          <t>foto-hero-3.jpg</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -731,23 +731,23 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Pendientes (estudio)</t>
+          <t>Hero slider 3</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>1200×1500 px
-≤400 KB</t>
+          <t>1920×1080 px
+≤300 KB</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
+          <t>Collar o pendientes en expositor de terciopelo oscuro. Iluminación de joyería de lujo.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
+          <t>Fine jewelry necklace with emeralds displayed on dark velvet, dramatic studio lighting, luxury brand photography, high contrast, ultra sharp details, elegant and minimal, 8K</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>images/home/home-slider-collares.jpg</t>
+          <t>foto-hero-3-modelo.jpg</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -767,23 +767,23 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Collares (estudio)</t>
+          <t>Hero slider 3 — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>1200×1500 px
-≤400 KB</t>
+          <t>1920×1080 px
+≤300 KB</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
+          <t>Se muestra al pasar el ratón sobre la foto 3, sin hacer clic. Mismo collar o pendientes puestos en modelo, fondo oscuro para mantener el ambiente.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
+          <t>Elegant woman wearing a fine emerald necklace, dramatic dark background, luxury brand editorial photography, high contrast, ultra sharp details, 8K</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>images/home/home-slider-pulseras.jpg</t>
+          <t>images/home/home-slider-anillos.jpg</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Pulseras (modelo)</t>
+          <t>Piezas que enamoran — Anillos (modelo)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -814,12 +814,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
+          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
+          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>images/home/home-destacado-1.jpg</t>
+          <t>images/home/home-slider-pendientes.jpg</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -839,23 +839,23 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 1</t>
+          <t>Piezas que enamoran — Pendientes (estudio)</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>images/home/home-destacado-2.jpg</t>
+          <t>images/home/home-slider-collares.jpg</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -875,23 +875,23 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 2</t>
+          <t>Piezas que enamoran — Collares (estudio)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>images/home/home-destacado-3.jpg</t>
+          <t>images/home/home-slider-pulseras.jpg</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -911,23 +911,23 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 3</t>
+          <t>Piezas que enamoran — Pulseras (modelo)</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>images/home/home-destacado-4.jpg</t>
+          <t>images/home/home-destacado-1.jpg</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 4</t>
+          <t>Piezas destacadas — pieza 1</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -973,33 +973,33 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>proceso-boceto.jpg</t>
+          <t>images/home/home-destacado-2.jpg</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Paso 1 — Boceto</t>
+          <t>Piezas destacadas — pieza 2</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -1009,33 +1009,33 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>proceso-materiales.jpg</t>
+          <t>images/home/home-destacado-3.jpg</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Paso 2 — Materiales</t>
+          <t>Piezas destacadas — pieza 3</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -1045,33 +1045,33 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>proceso-artesania.jpg</t>
+          <t>images/home/home-destacado-4.jpg</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Paso 3 — Artesanía</t>
+          <t>Piezas destacadas — pieza 4</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>proceso-entrega.jpg</t>
+          <t>proceso-boceto.jpg</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Paso 4 — Entrega</t>
+          <t>Paso 1 — Boceto</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1102,17 +1102,126 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
+          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="70" customHeight="1">
+      <c r="A20" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>proceso-materiales.jpg</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Paso 2 — Materiales</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="70" customHeight="1">
+      <c r="A21" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>proceso-artesania.jpg</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Paso 3 — Artesanía</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
+      <c r="A22" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>proceso-entrega.jpg</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Paso 4 — Entrega</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
           <t>Joya terminada en estuche o caja de regalo de lujo. Momento de entrega o presentación.</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen</t>
         </is>
@@ -1120,7 +1229,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Añadir 2ª foto en hover a las 3 imágenes del hero (#6)
Cada una de las 3 fotos del hero principal ahora muestra una segunda
imagen con un fundido suave al pasar el ratón por encima, sin
necesidad de hacer clic (foto-principal-modelo.jpg, foto-hero-2-modelo.jpg,
foto-hero-3-modelo.jpg). Pensado para alternar la foto de estudio con
la pieza puesta en modelo. Se actualiza el checklist de fotos con las
3 nuevas filas y sus prompts sugeridos.


Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G21"/>
+  <dimension ref="A2:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -613,7 +613,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>foto-hero-2.jpg</t>
+          <t>foto-principal-modelo.jpg</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Hero slider 2</t>
+          <t>Hero principal — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -634,12 +634,12 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Atelier o taller joyero: mesa de trabajo con herramientas artesanales, bocetos y materiales.</t>
+          <t>Se muestra al pasar el ratón sobre la foto principal, sin hacer clic. Misma joya puesta en modelo, para contrastar con la foto de estudio.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Luxury jewelry atelier workbench with golden tools, gemstones, sketches and magnifying glass, warm soft light, shallow depth of field, artisan craftsmanship, elegant editorial photography, 8K</t>
+          <t>The same exquisite gold diamond ring worn on an elegant female hand, editorial luxury jewelry campaign photography, soft natural light, neutral cream background, high-end style, ultra sharp, 8K</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>foto-hero-3.jpg</t>
+          <t>foto-hero-2.jpg</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Hero slider 3</t>
+          <t>Hero slider 2</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -670,12 +670,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Collar o pendientes en expositor de terciopelo oscuro. Iluminación de joyería de lujo.</t>
+          <t>Atelier o taller joyero: mesa de trabajo con herramientas artesanales, bocetos y materiales.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Fine jewelry necklace with emeralds displayed on dark velvet, dramatic studio lighting, luxury brand photography, high contrast, ultra sharp details, elegant and minimal, 8K</t>
+          <t>Luxury jewelry atelier workbench with golden tools, gemstones, sketches and magnifying glass, warm soft light, shallow depth of field, artisan craftsmanship, elegant editorial photography, 8K</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>images/home/home-slider-anillos.jpg</t>
+          <t>foto-hero-2-modelo.jpg</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -695,23 +695,23 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Anillos (modelo)</t>
+          <t>Hero slider 2 — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>1200×1500 px
-≤400 KB</t>
+          <t>1920×1080 px
+≤300 KB</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
+          <t>Se muestra al pasar el ratón sobre la foto 2, sin hacer clic. El anillo protagonista puesto en modelo, en vez de la vista del taller.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
+          <t>Close-up of a woman's hand wearing an elegant gold ring, editorial luxury jewelry campaign photography, warm soft light, shallow depth of field, elegant style, 8K</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>images/home/home-slider-pendientes.jpg</t>
+          <t>foto-hero-3.jpg</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -731,23 +731,23 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Pendientes (estudio)</t>
+          <t>Hero slider 3</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>1200×1500 px
-≤400 KB</t>
+          <t>1920×1080 px
+≤300 KB</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
+          <t>Collar o pendientes en expositor de terciopelo oscuro. Iluminación de joyería de lujo.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
+          <t>Fine jewelry necklace with emeralds displayed on dark velvet, dramatic studio lighting, luxury brand photography, high contrast, ultra sharp details, elegant and minimal, 8K</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>images/home/home-slider-collares.jpg</t>
+          <t>foto-hero-3-modelo.jpg</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -767,23 +767,23 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Collares (estudio)</t>
+          <t>Hero slider 3 — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>1200×1500 px
-≤400 KB</t>
+          <t>1920×1080 px
+≤300 KB</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
+          <t>Se muestra al pasar el ratón sobre la foto 3, sin hacer clic. Mismo collar o pendientes puestos en modelo, fondo oscuro para mantener el ambiente.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
+          <t>Elegant woman wearing a fine emerald necklace, dramatic dark background, luxury brand editorial photography, high contrast, ultra sharp details, 8K</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>images/home/home-slider-pulseras.jpg</t>
+          <t>images/home/home-slider-anillos.jpg</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Pulseras (modelo)</t>
+          <t>Piezas que enamoran — Anillos (modelo)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -814,12 +814,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
+          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
+          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>images/home/home-destacado-1.jpg</t>
+          <t>images/home/home-slider-pendientes.jpg</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -839,23 +839,23 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 1</t>
+          <t>Piezas que enamoran — Pendientes (estudio)</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>images/home/home-destacado-2.jpg</t>
+          <t>images/home/home-slider-collares.jpg</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -875,23 +875,23 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 2</t>
+          <t>Piezas que enamoran — Collares (estudio)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>images/home/home-destacado-3.jpg</t>
+          <t>images/home/home-slider-pulseras.jpg</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -911,23 +911,23 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 3</t>
+          <t>Piezas que enamoran — Pulseras (modelo)</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>images/home/home-destacado-4.jpg</t>
+          <t>images/home/home-destacado-1.jpg</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 4</t>
+          <t>Piezas destacadas — pieza 1</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -973,33 +973,33 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>proceso-boceto.jpg</t>
+          <t>images/home/home-destacado-2.jpg</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Paso 1 — Boceto</t>
+          <t>Piezas destacadas — pieza 2</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -1009,33 +1009,33 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>proceso-materiales.jpg</t>
+          <t>images/home/home-destacado-3.jpg</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Paso 2 — Materiales</t>
+          <t>Piezas destacadas — pieza 3</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -1045,33 +1045,33 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>proceso-artesania.jpg</t>
+          <t>images/home/home-destacado-4.jpg</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Paso 3 — Artesanía</t>
+          <t>Piezas destacadas — pieza 4</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>proceso-entrega.jpg</t>
+          <t>proceso-boceto.jpg</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Paso 4 — Entrega</t>
+          <t>Paso 1 — Boceto</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1102,17 +1102,126 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
+          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="70" customHeight="1">
+      <c r="A20" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>proceso-materiales.jpg</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Paso 2 — Materiales</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="70" customHeight="1">
+      <c r="A21" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>proceso-artesania.jpg</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Paso 3 — Artesanía</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
+      <c r="A22" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>proceso-entrega.jpg</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Paso 4 — Entrega</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
           <t>Joya terminada en estuche o caja de regalo de lujo. Momento de entrega o presentación.</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen</t>
         </is>
@@ -1120,7 +1229,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Añadir columnas de seguimiento al checklist de fotos
Añade "¿La has hecho?" (para que la marques tú manualmente con un
desplegable Sí/No) y "Subida a la web" (la actualizo yo cada hora
comprobando si el archivo ya existe en el repositorio).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,12 @@
       <i val="1"/>
       <color rgb="009A8FA5"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009A8FA5"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -147,6 +153,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -513,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G24"/>
+  <dimension ref="A2:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -523,6 +535,8 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="85" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -570,6 +584,16 @@
           <t>Prompt para Nanobanana</t>
         </is>
       </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>¿La has hecho?</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Subida a la web</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -606,6 +630,16 @@
           <t>Close-up of an exquisite gold ring with a sparkling diamond on elegant female hands with soft natural light, luxury jewelry photography, neutral cream background, high-end editorial style, ultra sharp, 8K</t>
         </is>
       </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="6" t="n">
@@ -642,6 +676,16 @@
           <t>The same exquisite gold diamond ring worn on an elegant female hand, editorial luxury jewelry campaign photography, soft natural light, neutral cream background, high-end style, ultra sharp, 8K</t>
         </is>
       </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -678,6 +722,16 @@
           <t>Luxury jewelry atelier workbench with golden tools, gemstones, sketches and magnifying glass, warm soft light, shallow depth of field, artisan craftsmanship, elegant editorial photography, 8K</t>
         </is>
       </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="6" t="n">
@@ -714,6 +768,16 @@
           <t>Close-up of a woman's hand wearing an elegant gold ring, editorial luxury jewelry campaign photography, warm soft light, shallow depth of field, elegant style, 8K</t>
         </is>
       </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -750,6 +814,16 @@
           <t>Fine jewelry necklace with emeralds displayed on dark velvet, dramatic studio lighting, luxury brand photography, high contrast, ultra sharp details, elegant and minimal, 8K</t>
         </is>
       </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -786,6 +860,16 @@
           <t>Elegant woman wearing a fine emerald necklace, dramatic dark background, luxury brand editorial photography, high contrast, ultra sharp details, 8K</t>
         </is>
       </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="70" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -822,6 +906,16 @@
           <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -858,6 +952,16 @@
           <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="70" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -894,6 +998,16 @@
           <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="70" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -930,6 +1044,16 @@
           <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="70" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -966,6 +1090,16 @@
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -1002,6 +1136,16 @@
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="70" customHeight="1">
       <c r="A17" s="3" t="n">
@@ -1038,6 +1182,16 @@
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -1074,6 +1228,16 @@
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="70" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -1110,6 +1274,16 @@
           <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
         </is>
       </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="70" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -1146,6 +1320,16 @@
           <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
         </is>
       </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="70" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -1182,6 +1366,16 @@
           <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
         </is>
       </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="70" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -1218,20 +1412,34 @@
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
-    </row>
-    <row r="23"/>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen</t>
+          <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen · "¿La has hecho?": marca Sí cuando tengas la foto lista · "Subida a la web": lo actualizo yo automáticamente cuando detecto el archivo subido en la carpeta correspondiente</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="H5:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No,Sí"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Añadir columnas de seguimiento al checklist de fotos (#7)
Añade "¿La has hecho?" (para que la marques tú manualmente con un
desplegable Sí/No) y "Subida a la web" (la actualizo yo cada hora
comprobando si el archivo ya existe en el repositorio).


Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,12 @@
       <i val="1"/>
       <color rgb="009A8FA5"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009A8FA5"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -147,6 +153,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -513,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G24"/>
+  <dimension ref="A2:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -523,6 +535,8 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="85" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -570,6 +584,16 @@
           <t>Prompt para Nanobanana</t>
         </is>
       </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>¿La has hecho?</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Subida a la web</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -606,6 +630,16 @@
           <t>Close-up of an exquisite gold ring with a sparkling diamond on elegant female hands with soft natural light, luxury jewelry photography, neutral cream background, high-end editorial style, ultra sharp, 8K</t>
         </is>
       </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="6" t="n">
@@ -642,6 +676,16 @@
           <t>The same exquisite gold diamond ring worn on an elegant female hand, editorial luxury jewelry campaign photography, soft natural light, neutral cream background, high-end style, ultra sharp, 8K</t>
         </is>
       </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -678,6 +722,16 @@
           <t>Luxury jewelry atelier workbench with golden tools, gemstones, sketches and magnifying glass, warm soft light, shallow depth of field, artisan craftsmanship, elegant editorial photography, 8K</t>
         </is>
       </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="6" t="n">
@@ -714,6 +768,16 @@
           <t>Close-up of a woman's hand wearing an elegant gold ring, editorial luxury jewelry campaign photography, warm soft light, shallow depth of field, elegant style, 8K</t>
         </is>
       </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -750,6 +814,16 @@
           <t>Fine jewelry necklace with emeralds displayed on dark velvet, dramatic studio lighting, luxury brand photography, high contrast, ultra sharp details, elegant and minimal, 8K</t>
         </is>
       </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -786,6 +860,16 @@
           <t>Elegant woman wearing a fine emerald necklace, dramatic dark background, luxury brand editorial photography, high contrast, ultra sharp details, 8K</t>
         </is>
       </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="70" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -822,6 +906,16 @@
           <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -858,6 +952,16 @@
           <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="70" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -894,6 +998,16 @@
           <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="70" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -930,6 +1044,16 @@
           <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="70" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -966,6 +1090,16 @@
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -1002,6 +1136,16 @@
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="70" customHeight="1">
       <c r="A17" s="3" t="n">
@@ -1038,6 +1182,16 @@
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -1074,6 +1228,16 @@
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="70" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -1110,6 +1274,16 @@
           <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
         </is>
       </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="70" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -1146,6 +1320,16 @@
           <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
         </is>
       </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="70" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -1182,6 +1366,16 @@
           <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
         </is>
       </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="70" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -1218,20 +1412,34 @@
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
-    </row>
-    <row r="23"/>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen</t>
+          <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen · "¿La has hecho?": marca Sí cuando tengas la foto lista · "Subida a la web": lo actualizo yo automáticamente cuando detecto el archivo subido en la carpeta correspondiente</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="H5:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No,Sí"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Separar nombre de archivo y carpeta destino en el checklist
La columna "Archivo" incluía rutas como "images/home/foto.jpg", que
Windows rechaza al guardar (no admite "/" en el nombre). Ahora
"Archivo" solo tiene el nombre del archivo y una nueva columna
"Carpeta destino" indica dónde guardarlo (Raíz del proyecto /
images/home).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,8 +65,31 @@
       <color rgb="002E7D32"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B48FC8"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A1520"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009A8FA5"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -98,8 +121,23 @@
         <fgColor rgb="FFEDE0F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004A3F52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F2FC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -122,11 +160,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D4B8E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D4B8E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D4B8E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D4B8E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -166,6 +218,39 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -533,17 +618,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:I24"/>
+  <dimension ref="A2:J24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="11" min="1" max="1"/>
-    <col width="32" customWidth="1" style="11" min="2" max="2"/>
-    <col width="20" customWidth="1" style="11" min="3" max="3"/>
-    <col width="18" customWidth="1" style="11" min="4" max="4"/>
-    <col width="14" customWidth="1" style="11" min="5" max="5"/>
-    <col width="55" customWidth="1" style="11" min="6" max="6"/>
-    <col width="85" customWidth="1" style="11" min="7" max="7"/>
-    <col width="16" customWidth="1" style="11" min="8" max="9"/>
+    <col width="26" customWidth="1" style="11" min="2" max="2"/>
+    <col width="16" customWidth="1" style="11" min="3" max="3"/>
+    <col width="20" customWidth="1" style="11" min="4" max="4"/>
+    <col width="30" customWidth="1" style="11" min="5" max="5"/>
+    <col width="14" customWidth="1" style="11" min="6" max="6"/>
+    <col width="55" customWidth="1" style="11" min="7" max="7"/>
+    <col width="85" customWidth="1" style="11" min="8" max="9"/>
+    <col width="16" customWidth="1" style="11" min="9" max="9"/>
+    <col width="16" customWidth="1" style="11" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="11"/>
@@ -556,875 +643,970 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="11"/>
     <row r="4" ht="27.95" customHeight="1" s="11">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Archivo</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Carpeta destino</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Página</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Sección</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Medidas</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>Descripción / Contenido</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="H4" s="15" t="inlineStr">
         <is>
           <t>Prompt para Nanobanana</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="I4" s="15" t="inlineStr">
         <is>
           <t>¿La has hecho?</t>
         </is>
       </c>
-      <c r="I4" s="1" t="inlineStr">
+      <c r="J4" s="15" t="inlineStr">
         <is>
           <t>Subida a la web</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="69.95" customHeight="1" s="11">
-      <c r="A5" s="2" t="n">
+    <row r="5" ht="70" customHeight="1" s="11">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>foto-principal.jpg</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Hero principal</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Joya estrella sobre fondo neutro o manos de mujer sosteniéndola. Imagen impactante, elegante, con mucha luz.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>Close-up of an exquisite gold ring with a sparkling diamond on elegant female hands with soft natural light, luxury jewelry photography, neutral cream background, high-end editorial style, ultra sharp, 8K</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="I5" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="J5" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="69.95" customHeight="1" s="11">
-      <c r="A6" s="5" t="n">
+    <row r="6" ht="70" customHeight="1" s="11">
+      <c r="A6" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>foto-principal-modelo.jpg</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>Hero principal — 2ª foto en hover (modelo)</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>Se muestra al pasar el ratón sobre la foto principal, sin hacer clic. Misma joya puesta en modelo, para contrastar con la foto de estudio.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>The same exquisite gold diamond ring worn on an elegant female hand, editorial luxury jewelry campaign photography, soft natural light, neutral cream background, high-end style, ultra sharp, 8K</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="I6" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="J6" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="69.95" customHeight="1" s="11">
-      <c r="A7" s="2" t="n">
+    <row r="7" ht="70" customHeight="1" s="11">
+      <c r="A7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>foto-hero-2.jpg</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Hero slider 2</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>Atelier o taller joyero: mesa de trabajo con herramientas artesanales, bocetos y materiales.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>Luxury jewelry atelier workbench with golden tools, gemstones, sketches and magnifying glass, warm soft light, shallow depth of field, artisan craftsmanship, elegant editorial photography, 8K</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="I7" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I7" s="13" t="inlineStr">
+      <c r="J7" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="69.95" customHeight="1" s="11">
-      <c r="A8" s="5" t="n">
+    <row r="8" ht="70" customHeight="1" s="11">
+      <c r="A8" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>foto-hero-2-modelo.jpg</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Hero slider 2 — 2ª foto en hover (modelo)</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>Se muestra al pasar el ratón sobre la foto 2, sin hacer clic. El anillo protagonista puesto en modelo, en vez de la vista del taller.</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>Close-up of a woman's hand wearing an elegant gold ring, editorial luxury jewelry campaign photography, warm soft light, shallow depth of field, elegant style, 8K</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="I8" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr">
+      <c r="J8" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="69.95" customHeight="1" s="11">
-      <c r="A9" s="2" t="n">
+    <row r="9" ht="70" customHeight="1" s="11">
+      <c r="A9" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>foto-hero-3.jpg</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Hero slider 3</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>Collar o pendientes en expositor de terciopelo oscuro. Iluminación de joyería de lujo.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>Fine jewelry necklace with emeralds displayed on dark velvet, dramatic studio lighting, luxury brand photography, high contrast, ultra sharp details, elegant and minimal, 8K</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="I9" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr">
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="69.95" customHeight="1" s="11">
-      <c r="A10" s="5" t="n">
+    <row r="10" ht="70" customHeight="1" s="11">
+      <c r="A10" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>foto-hero-3-modelo.jpg</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>Hero slider 3 — 2ª foto en hover (modelo)</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="F10" s="22" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Se muestra al pasar el ratón sobre la foto 3, sin hacer clic. Mismo collar o pendientes puestos en modelo, fondo oscuro para mantener el ambiente.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>Elegant woman wearing a fine emerald necklace, dramatic dark background, luxury brand editorial photography, high contrast, ultra sharp details, 8K</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="I10" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="69.95" customHeight="1" s="11">
-      <c r="A11" s="2" t="n">
+    <row r="11" ht="70" customHeight="1" s="11">
+      <c r="A11" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>images/home/home-slider-anillos.jpg</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>home-slider-anillos.jpg</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>Piezas que enamoran — Anillos (modelo)</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>1200×1500 px
 ≤400 KB</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="69.95" customHeight="1" s="11">
-      <c r="A12" s="5" t="n">
+      <c r="I11" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1" s="11">
+      <c r="A12" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>images/home/home-slider-pendientes.jpg</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>home-slider-pendientes.jpg</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>Piezas que enamoran — Pendientes (estudio)</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="F12" s="22" t="inlineStr">
         <is>
           <t>1200×1500 px
 ≤400 KB</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="H12" s="21" t="inlineStr">
         <is>
           <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="69.95" customHeight="1" s="11">
-      <c r="A13" s="2" t="n">
+      <c r="I12" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J12" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1" s="11">
+      <c r="A13" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>images/home/home-slider-collares.jpg</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>home-slider-collares.jpg</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>Piezas que enamoran — Collares (estudio)</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>1200×1500 px
 ≤400 KB</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
         <is>
           <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="69.95" customHeight="1" s="11">
-      <c r="A14" s="5" t="n">
+      <c r="I13" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="70" customHeight="1" s="11">
+      <c r="A14" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>images/home/home-slider-pulseras.jpg</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>home-slider-pulseras.jpg</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>Piezas que enamoran — Pulseras (modelo)</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="F14" s="22" t="inlineStr">
         <is>
           <t>1200×1500 px
 ≤400 KB</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I14" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="69.95" customHeight="1" s="11">
-      <c r="A15" s="2" t="n">
+      <c r="I14" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J14" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="70" customHeight="1" s="11">
+      <c r="A15" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>images/home/home-destacado-1.jpg</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>home-destacado-1.jpg</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>Piezas destacadas — pieza 1</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" s="17" t="inlineStr">
         <is>
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="69.95" customHeight="1" s="11">
-      <c r="A16" s="5" t="n">
+      <c r="I15" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J15" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1" s="11">
+      <c r="A16" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>images/home/home-destacado-2.jpg</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>home-destacado-2.jpg</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>Piezas destacadas — pieza 2</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="F16" s="22" t="inlineStr">
         <is>
           <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="69.95" customHeight="1" s="11">
-      <c r="A17" s="2" t="n">
+      <c r="I16" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1" s="11">
+      <c r="A17" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>images/home/home-destacado-3.jpg</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>home-destacado-3.jpg</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>Piezas destacadas — pieza 3</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
         <is>
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="69.95" customHeight="1" s="11">
-      <c r="A18" s="5" t="n">
+      <c r="I17" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J17" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1" s="11">
+      <c r="A18" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>images/home/home-destacado-4.jpg</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>home-destacado-4.jpg</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>Piezas destacadas — pieza 4</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="F18" s="22" t="inlineStr">
         <is>
           <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="H18" s="21" t="inlineStr">
         <is>
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="69.95" customHeight="1" s="11">
-      <c r="A19" s="2" t="n">
+      <c r="I18" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J18" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="70" customHeight="1" s="11">
+      <c r="A19" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>proceso-boceto.jpg</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="E19" s="18" t="inlineStr">
         <is>
           <t>Paso 1 — Boceto</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="69.95" customHeight="1" s="11">
-      <c r="A20" s="5" t="n">
+      <c r="I19" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J19" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="70" customHeight="1" s="11">
+      <c r="A20" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>proceso-materiales.jpg</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>Paso 2 — Materiales</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="F20" s="22" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="G20" s="21" t="inlineStr">
         <is>
           <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="H20" s="21" t="inlineStr">
         <is>
           <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I20" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="69.95" customHeight="1" s="11">
-      <c r="A21" s="2" t="n">
+      <c r="I20" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J20" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="70" customHeight="1" s="11">
+      <c r="A21" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>proceso-artesania.jpg</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="E21" s="18" t="inlineStr">
         <is>
           <t>Paso 3 — Artesanía</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="F21" s="18" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" s="17" t="inlineStr">
         <is>
           <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="69.95" customHeight="1" s="11">
-      <c r="A22" s="5" t="n">
+      <c r="I21" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J21" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1" s="11">
+      <c r="A22" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>proceso-entrega.jpg</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="E22" s="22" t="inlineStr">
         <is>
           <t>Paso 4 — Entrega</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="F22" s="22" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="G22" s="21" t="inlineStr">
         <is>
           <t>Joya terminada en estuche o caja de regalo de lujo. Momento de entrega o presentación.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="H22" s="21" t="inlineStr">
         <is>
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
+      <c r="I22" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J22" s="25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1433,17 +1615,20 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen · "¿La has hecho?": marca Sí cuando tengas la foto lista · "Subida a la web": lo actualizo yo automáticamente cuando detecto el archivo subido en la carpeta correspondiente</t>
+          <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen · "¿La has hecho?": marca Sí cuando tengas la foto lista · "Subida a la web": lo actualizo yo automáticamente cuando detecto el archivo subido en la carpeta correspondiente · "Carpeta destino": dónde va cada archivo dentro del proyecto (raíz, o dentro de la carpeta images/home)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="H5:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No,Sí"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I5:I22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Sí"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Separar nombre de archivo y carpeta destino en el checklist (#12)
La columna "Archivo" incluía rutas como "images/home/foto.jpg", que
Windows rechaza al guardar (no admite "/" en el nombre). Ahora
"Archivo" solo tiene el nombre del archivo y una nueva columna
"Carpeta destino" indica dónde guardarlo (Raíz del proyecto /
images/home).


Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,8 +65,31 @@
       <color rgb="002E7D32"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B48FC8"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A1520"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009A8FA5"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -98,8 +121,23 @@
         <fgColor rgb="FFEDE0F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004A3F52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F2FC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -122,11 +160,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D4B8E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D4B8E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D4B8E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D4B8E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -166,6 +218,39 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -533,17 +618,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:I24"/>
+  <dimension ref="A2:J24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="11" min="1" max="1"/>
-    <col width="32" customWidth="1" style="11" min="2" max="2"/>
-    <col width="20" customWidth="1" style="11" min="3" max="3"/>
-    <col width="18" customWidth="1" style="11" min="4" max="4"/>
-    <col width="14" customWidth="1" style="11" min="5" max="5"/>
-    <col width="55" customWidth="1" style="11" min="6" max="6"/>
-    <col width="85" customWidth="1" style="11" min="7" max="7"/>
-    <col width="16" customWidth="1" style="11" min="8" max="9"/>
+    <col width="26" customWidth="1" style="11" min="2" max="2"/>
+    <col width="16" customWidth="1" style="11" min="3" max="3"/>
+    <col width="20" customWidth="1" style="11" min="4" max="4"/>
+    <col width="30" customWidth="1" style="11" min="5" max="5"/>
+    <col width="14" customWidth="1" style="11" min="6" max="6"/>
+    <col width="55" customWidth="1" style="11" min="7" max="7"/>
+    <col width="85" customWidth="1" style="11" min="8" max="9"/>
+    <col width="16" customWidth="1" style="11" min="9" max="9"/>
+    <col width="16" customWidth="1" style="11" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="11"/>
@@ -556,875 +643,970 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="11"/>
     <row r="4" ht="27.95" customHeight="1" s="11">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Archivo</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Carpeta destino</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Página</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Sección</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Medidas</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>Descripción / Contenido</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="H4" s="15" t="inlineStr">
         <is>
           <t>Prompt para Nanobanana</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="I4" s="15" t="inlineStr">
         <is>
           <t>¿La has hecho?</t>
         </is>
       </c>
-      <c r="I4" s="1" t="inlineStr">
+      <c r="J4" s="15" t="inlineStr">
         <is>
           <t>Subida a la web</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="69.95" customHeight="1" s="11">
-      <c r="A5" s="2" t="n">
+    <row r="5" ht="70" customHeight="1" s="11">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>foto-principal.jpg</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Hero principal</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Joya estrella sobre fondo neutro o manos de mujer sosteniéndola. Imagen impactante, elegante, con mucha luz.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>Close-up of an exquisite gold ring with a sparkling diamond on elegant female hands with soft natural light, luxury jewelry photography, neutral cream background, high-end editorial style, ultra sharp, 8K</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="I5" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="J5" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="69.95" customHeight="1" s="11">
-      <c r="A6" s="5" t="n">
+    <row r="6" ht="70" customHeight="1" s="11">
+      <c r="A6" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>foto-principal-modelo.jpg</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>Hero principal — 2ª foto en hover (modelo)</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>Se muestra al pasar el ratón sobre la foto principal, sin hacer clic. Misma joya puesta en modelo, para contrastar con la foto de estudio.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>The same exquisite gold diamond ring worn on an elegant female hand, editorial luxury jewelry campaign photography, soft natural light, neutral cream background, high-end style, ultra sharp, 8K</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="I6" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="J6" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="69.95" customHeight="1" s="11">
-      <c r="A7" s="2" t="n">
+    <row r="7" ht="70" customHeight="1" s="11">
+      <c r="A7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>foto-hero-2.jpg</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Hero slider 2</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>Atelier o taller joyero: mesa de trabajo con herramientas artesanales, bocetos y materiales.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>Luxury jewelry atelier workbench with golden tools, gemstones, sketches and magnifying glass, warm soft light, shallow depth of field, artisan craftsmanship, elegant editorial photography, 8K</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="I7" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I7" s="13" t="inlineStr">
+      <c r="J7" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="69.95" customHeight="1" s="11">
-      <c r="A8" s="5" t="n">
+    <row r="8" ht="70" customHeight="1" s="11">
+      <c r="A8" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>foto-hero-2-modelo.jpg</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Hero slider 2 — 2ª foto en hover (modelo)</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>Se muestra al pasar el ratón sobre la foto 2, sin hacer clic. El anillo protagonista puesto en modelo, en vez de la vista del taller.</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>Close-up of a woman's hand wearing an elegant gold ring, editorial luxury jewelry campaign photography, warm soft light, shallow depth of field, elegant style, 8K</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="I8" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr">
+      <c r="J8" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="69.95" customHeight="1" s="11">
-      <c r="A9" s="2" t="n">
+    <row r="9" ht="70" customHeight="1" s="11">
+      <c r="A9" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>foto-hero-3.jpg</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Hero slider 3</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>Collar o pendientes en expositor de terciopelo oscuro. Iluminación de joyería de lujo.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>Fine jewelry necklace with emeralds displayed on dark velvet, dramatic studio lighting, luxury brand photography, high contrast, ultra sharp details, elegant and minimal, 8K</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="I9" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr">
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="69.95" customHeight="1" s="11">
-      <c r="A10" s="5" t="n">
+    <row r="10" ht="70" customHeight="1" s="11">
+      <c r="A10" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>foto-hero-3-modelo.jpg</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>Hero slider 3 — 2ª foto en hover (modelo)</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="F10" s="22" t="inlineStr">
         <is>
           <t>1920×1080 px
 ≤300 KB</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Se muestra al pasar el ratón sobre la foto 3, sin hacer clic. Mismo collar o pendientes puestos en modelo, fondo oscuro para mantener el ambiente.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>Elegant woman wearing a fine emerald necklace, dramatic dark background, luxury brand editorial photography, high contrast, ultra sharp details, 8K</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="I10" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="69.95" customHeight="1" s="11">
-      <c r="A11" s="2" t="n">
+    <row r="11" ht="70" customHeight="1" s="11">
+      <c r="A11" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>images/home/home-slider-anillos.jpg</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>home-slider-anillos.jpg</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>Piezas que enamoran — Anillos (modelo)</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>1200×1500 px
 ≤400 KB</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="69.95" customHeight="1" s="11">
-      <c r="A12" s="5" t="n">
+      <c r="I11" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1" s="11">
+      <c r="A12" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>images/home/home-slider-pendientes.jpg</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>home-slider-pendientes.jpg</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>Piezas que enamoran — Pendientes (estudio)</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="F12" s="22" t="inlineStr">
         <is>
           <t>1200×1500 px
 ≤400 KB</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="H12" s="21" t="inlineStr">
         <is>
           <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="69.95" customHeight="1" s="11">
-      <c r="A13" s="2" t="n">
+      <c r="I12" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J12" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1" s="11">
+      <c r="A13" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>images/home/home-slider-collares.jpg</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>home-slider-collares.jpg</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>Piezas que enamoran — Collares (estudio)</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>1200×1500 px
 ≤400 KB</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
         <is>
           <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="69.95" customHeight="1" s="11">
-      <c r="A14" s="5" t="n">
+      <c r="I13" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="70" customHeight="1" s="11">
+      <c r="A14" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>images/home/home-slider-pulseras.jpg</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>home-slider-pulseras.jpg</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>Piezas que enamoran — Pulseras (modelo)</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="F14" s="22" t="inlineStr">
         <is>
           <t>1200×1500 px
 ≤400 KB</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I14" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="69.95" customHeight="1" s="11">
-      <c r="A15" s="2" t="n">
+      <c r="I14" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J14" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="70" customHeight="1" s="11">
+      <c r="A15" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>images/home/home-destacado-1.jpg</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>home-destacado-1.jpg</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>Piezas destacadas — pieza 1</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" s="17" t="inlineStr">
         <is>
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="69.95" customHeight="1" s="11">
-      <c r="A16" s="5" t="n">
+      <c r="I15" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J15" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1" s="11">
+      <c r="A16" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>images/home/home-destacado-2.jpg</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>home-destacado-2.jpg</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>Piezas destacadas — pieza 2</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="F16" s="22" t="inlineStr">
         <is>
           <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="69.95" customHeight="1" s="11">
-      <c r="A17" s="2" t="n">
+      <c r="I16" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1" s="11">
+      <c r="A17" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>images/home/home-destacado-3.jpg</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>home-destacado-3.jpg</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>Piezas destacadas — pieza 3</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
         <is>
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="69.95" customHeight="1" s="11">
-      <c r="A18" s="5" t="n">
+      <c r="I17" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J17" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1" s="11">
+      <c r="A18" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>images/home/home-destacado-4.jpg</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>home-destacado-4.jpg</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>Piezas destacadas — pieza 4</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="F18" s="22" t="inlineStr">
         <is>
           <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="H18" s="21" t="inlineStr">
         <is>
           <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="69.95" customHeight="1" s="11">
-      <c r="A19" s="2" t="n">
+      <c r="I18" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J18" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="70" customHeight="1" s="11">
+      <c r="A19" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>proceso-boceto.jpg</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="E19" s="18" t="inlineStr">
         <is>
           <t>Paso 1 — Boceto</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="69.95" customHeight="1" s="11">
-      <c r="A20" s="5" t="n">
+      <c r="I19" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J19" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="70" customHeight="1" s="11">
+      <c r="A20" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>proceso-materiales.jpg</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>Paso 2 — Materiales</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="F20" s="22" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="G20" s="21" t="inlineStr">
         <is>
           <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="H20" s="21" t="inlineStr">
         <is>
           <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I20" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="69.95" customHeight="1" s="11">
-      <c r="A21" s="2" t="n">
+      <c r="I20" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J20" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="70" customHeight="1" s="11">
+      <c r="A21" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>proceso-artesania.jpg</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="E21" s="18" t="inlineStr">
         <is>
           <t>Paso 3 — Artesanía</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="F21" s="18" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" s="17" t="inlineStr">
         <is>
           <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="69.95" customHeight="1" s="11">
-      <c r="A22" s="5" t="n">
+      <c r="I21" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J21" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1" s="11">
+      <c r="A22" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>proceso-entrega.jpg</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="E22" s="22" t="inlineStr">
         <is>
           <t>Paso 4 — Entrega</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="F22" s="22" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="G22" s="21" t="inlineStr">
         <is>
           <t>Joya terminada en estuche o caja de regalo de lujo. Momento de entrega o presentación.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="H22" s="21" t="inlineStr">
         <is>
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
+      <c r="I22" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J22" s="25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1433,17 +1615,20 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen · "¿La has hecho?": marca Sí cuando tengas la foto lista · "Subida a la web": lo actualizo yo automáticamente cuando detecto el archivo subido en la carpeta correspondiente</t>
+          <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen · "¿La has hecho?": marca Sí cuando tengas la foto lista · "Subida a la web": lo actualizo yo automáticamente cuando detecto el archivo subido en la carpeta correspondiente · "Carpeta destino": dónde va cada archivo dentro del proyecto (raíz, o dentro de la carpeta images/home)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="H5:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No,Sí"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I5:I22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Sí"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Añadir foto de estudio y de modelo a cada sección del slider de piezas
Las 4 secciones del slider "Piezas que enamoran" (Anillos, Pendientes,
Collares, Pulseras) ahora tienen 2 fotos cada una, igual que el hero:
foto de estudio por defecto y foto con modelo en fundido al pasar el
ratón (piezas-photo-base / piezas-photo-alt). La etiqueta de cada
sección pasa a blanco en el hover, en vez de tener un color fijo.

Se actualiza el checklist con las 4 fotos "modelo" que faltaban
(8 filas en total para el slider) y se corrige un desplegable de
"¿La has hecho?" que había quedado mal referenciado sobre la columna
del prompt tras el cambio de columnas anterior.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,6 +87,12 @@
       <b val="1"/>
       <color rgb="009A8FA5"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="009A8FA5"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="10">
@@ -178,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -252,6 +258,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -618,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J24"/>
+  <dimension ref="A2:J28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="11" min="1" max="1"/>
@@ -1021,7 +1030,7 @@
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Anillos (modelo)</t>
+          <t>Piezas que enamoran — Anillos (estudio)</t>
         </is>
       </c>
       <c r="F11" s="18" t="inlineStr">
@@ -1032,12 +1041,12 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
+          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Anillos en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
+          <t>Elegant gold rings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
       <c r="I11" s="24" t="inlineStr">
@@ -1057,7 +1066,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>home-slider-pendientes.jpg</t>
+          <t>home-slider-anillos-modelo.jpg</t>
         </is>
       </c>
       <c r="C12" s="22" t="inlineStr">
@@ -1072,7 +1081,7 @@
       </c>
       <c r="E12" s="22" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Pendientes (estudio)</t>
+          <t>Piezas que enamoran — Anillos — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="F12" s="22" t="inlineStr">
@@ -1083,12 +1092,12 @@
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
+          <t>Se muestra al pasar el ratón sobre la foto de Anillos, sin hacer clic. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
         </is>
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
-          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
+          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
       <c r="I12" s="25" t="inlineStr">
@@ -1108,7 +1117,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>home-slider-collares.jpg</t>
+          <t>home-slider-pendientes.jpg</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1123,7 +1132,7 @@
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Collares (estudio)</t>
+          <t>Piezas que enamoran — Pendientes (estudio)</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
@@ -1134,12 +1143,12 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
+          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
-          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
+          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
       <c r="I13" s="24" t="inlineStr">
@@ -1159,7 +1168,7 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>home-slider-pulseras.jpg</t>
+          <t>home-slider-pendientes-modelo.jpg</t>
         </is>
       </c>
       <c r="C14" s="22" t="inlineStr">
@@ -1174,7 +1183,7 @@
       </c>
       <c r="E14" s="22" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Pulseras (modelo)</t>
+          <t>Piezas que enamoran — Pendientes — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="F14" s="22" t="inlineStr">
@@ -1185,12 +1194,12 @@
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
+          <t>Se muestra al pasar el ratón sobre la foto de Pendientes, sin hacer clic. Modelo llevando los pendientes, primer plano de rostro y oreja.</t>
         </is>
       </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
-          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
+          <t>Close-up of a woman's face wearing elegant gold earrings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
       <c r="I14" s="25" t="inlineStr">
@@ -1210,7 +1219,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>home-destacado-1.jpg</t>
+          <t>home-slider-collares.jpg</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -1225,23 +1234,23 @@
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 1</t>
+          <t>Piezas que enamoran — Collares (estudio)</t>
         </is>
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
       <c r="I15" s="24" t="inlineStr">
@@ -1261,7 +1270,7 @@
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>home-destacado-2.jpg</t>
+          <t>home-slider-collares-modelo.jpg</t>
         </is>
       </c>
       <c r="C16" s="22" t="inlineStr">
@@ -1276,23 +1285,23 @@
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 2</t>
+          <t>Piezas que enamoran — Collares — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="F16" s="22" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Se muestra al pasar el ratón sobre la foto de Collares, sin hacer clic. Modelo llevando el collar, plano de escote y cuello.</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Elegant woman wearing a fine gold necklace, close-up of neckline and collarbone, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
       <c r="I16" s="25" t="inlineStr">
@@ -1312,7 +1321,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>home-destacado-3.jpg</t>
+          <t>home-slider-pulseras.jpg</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1327,23 +1336,23 @@
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 3</t>
+          <t>Piezas que enamoran — Pulseras (estudio)</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Pulseras en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Elegant gold bracelets arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
       <c r="I17" s="24" t="inlineStr">
@@ -1363,7 +1372,7 @@
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>home-destacado-4.jpg</t>
+          <t>home-slider-pulseras-modelo.jpg</t>
         </is>
       </c>
       <c r="C18" s="22" t="inlineStr">
@@ -1378,23 +1387,23 @@
       </c>
       <c r="E18" s="22" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 4</t>
+          <t>Piezas que enamoran — Pulseras — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="F18" s="22" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Se muestra al pasar el ratón sobre la foto de Pulseras, sin hacer clic. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
       <c r="I18" s="25" t="inlineStr">
@@ -1414,38 +1423,38 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>proceso-boceto.jpg</t>
+          <t>home-destacado-1.jpg</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Raíz del proyecto</t>
+          <t>images/home</t>
         </is>
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
         <is>
-          <t>Paso 1 — Boceto</t>
+          <t>Piezas destacadas — pieza 1</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="H19" s="17" t="inlineStr">
         <is>
-          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
       <c r="I19" s="24" t="inlineStr">
@@ -1465,38 +1474,38 @@
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>proceso-materiales.jpg</t>
+          <t>home-destacado-2.jpg</t>
         </is>
       </c>
       <c r="C20" s="22" t="inlineStr">
         <is>
-          <t>Raíz del proyecto</t>
+          <t>images/home</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="E20" s="22" t="inlineStr">
         <is>
-          <t>Paso 2 — Materiales</t>
+          <t>Piezas destacadas — pieza 2</t>
         </is>
       </c>
       <c r="F20" s="22" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="G20" s="21" t="inlineStr">
         <is>
-          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="H20" s="21" t="inlineStr">
         <is>
-          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
       <c r="I20" s="25" t="inlineStr">
@@ -1516,38 +1525,38 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>proceso-artesania.jpg</t>
+          <t>home-destacado-3.jpg</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Raíz del proyecto</t>
+          <t>images/home</t>
         </is>
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
         <is>
-          <t>Paso 3 — Artesanía</t>
+          <t>Piezas destacadas — pieza 3</t>
         </is>
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
-          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
       <c r="I21" s="24" t="inlineStr">
@@ -1567,53 +1576,257 @@
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>proceso-entrega.jpg</t>
+          <t>home-destacado-4.jpg</t>
         </is>
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>Piezas destacadas — pieza 4</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>800×1000 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="inlineStr">
+        <is>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+        </is>
+      </c>
+      <c r="I22" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J22" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="70" customHeight="1" s="11">
+      <c r="A23" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>proceso-boceto.jpg</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
           <t>Raíz del proyecto</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
-        <is>
-          <t>Paso 4 — Entrega</t>
-        </is>
-      </c>
-      <c r="F22" s="22" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Paso 1 — Boceto</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="G22" s="21" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J23" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="70" customHeight="1" s="11">
+      <c r="A24" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>proceso-materiales.jpg</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Paso 2 — Materiales</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="G24" s="21" t="inlineStr">
+        <is>
+          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+        </is>
+      </c>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+        </is>
+      </c>
+      <c r="I24" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J24" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="70" customHeight="1" s="11">
+      <c r="A25" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>proceso-artesania.jpg</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Paso 3 — Artesanía</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+        </is>
+      </c>
+      <c r="I25" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J25" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="70" customHeight="1" s="11">
+      <c r="A26" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>proceso-entrega.jpg</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>Paso 4 — Entrega</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="G26" s="21" t="inlineStr">
         <is>
           <t>Joya terminada en estuche o caja de regalo de lujo. Momento de entrega o presentación.</t>
         </is>
       </c>
-      <c r="H22" s="21" t="inlineStr">
+      <c r="H26" s="21" t="inlineStr">
         <is>
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
-      <c r="I22" s="25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J22" s="25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="I26" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J26" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen · "¿La has hecho?": marca Sí cuando tengas la foto lista · "Subida a la web": lo actualizo yo automáticamente cuando detecto el archivo subido en la carpeta correspondiente · "Carpeta destino": dónde va cada archivo dentro del proyecto (raíz, o dentro de la carpeta images/home)</t>
         </is>
@@ -1621,14 +1834,11 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A28:J28"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation sqref="H5:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Sí"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I5:I22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="1">
+    <dataValidation sqref="I5:I26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Sí"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Añadir foto de estudio y de modelo a cada sección del slider de piezas (#13)
Las 4 secciones del slider "Piezas que enamoran" (Anillos, Pendientes,
Collares, Pulseras) ahora tienen 2 fotos cada una, igual que el hero:
foto de estudio por defecto y foto con modelo en fundido al pasar el
ratón (piezas-photo-base / piezas-photo-alt). La etiqueta de cada
sección pasa a blanco en el hover, en vez de tener un color fijo.

Se actualiza el checklist con las 4 fotos "modelo" que faltaban
(8 filas en total para el slider) y se corrige un desplegable de
"¿La has hecho?" que había quedado mal referenciado sobre la columna
del prompt tras el cambio de columnas anterior.


Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,6 +87,12 @@
       <b val="1"/>
       <color rgb="009A8FA5"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="009A8FA5"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="10">
@@ -178,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -252,6 +258,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -618,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J24"/>
+  <dimension ref="A2:J28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="11" min="1" max="1"/>
@@ -1021,7 +1030,7 @@
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Anillos (modelo)</t>
+          <t>Piezas que enamoran — Anillos (estudio)</t>
         </is>
       </c>
       <c r="F11" s="18" t="inlineStr">
@@ -1032,12 +1041,12 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
+          <t>Mitad izquierda de la 1ª fila del slider a pantalla completa. Anillos en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
+          <t>Elegant gold rings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
       <c r="I11" s="24" t="inlineStr">
@@ -1057,7 +1066,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>home-slider-pendientes.jpg</t>
+          <t>home-slider-anillos-modelo.jpg</t>
         </is>
       </c>
       <c r="C12" s="22" t="inlineStr">
@@ -1072,7 +1081,7 @@
       </c>
       <c r="E12" s="22" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Pendientes (estudio)</t>
+          <t>Piezas que enamoran — Anillos — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="F12" s="22" t="inlineStr">
@@ -1083,12 +1092,12 @@
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
+          <t>Se muestra al pasar el ratón sobre la foto de Anillos, sin hacer clic. Modelo llevando anillos, plano de mano o muñeca en primer plano.</t>
         </is>
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
-          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
+          <t>Close-up of a woman's hand and wrist wearing elegant gold rings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
       <c r="I12" s="25" t="inlineStr">
@@ -1108,7 +1117,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>home-slider-collares.jpg</t>
+          <t>home-slider-pendientes.jpg</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1123,7 +1132,7 @@
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Collares (estudio)</t>
+          <t>Piezas que enamoran — Pendientes (estudio)</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
@@ -1134,12 +1143,12 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
+          <t>Mitad derecha de la 1ª fila del slider a pantalla completa. Pendientes en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
-          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
+          <t>Elegant gold earrings arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
       <c r="I13" s="24" t="inlineStr">
@@ -1159,7 +1168,7 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>home-slider-pulseras.jpg</t>
+          <t>home-slider-pendientes-modelo.jpg</t>
         </is>
       </c>
       <c r="C14" s="22" t="inlineStr">
@@ -1174,7 +1183,7 @@
       </c>
       <c r="E14" s="22" t="inlineStr">
         <is>
-          <t>Piezas que enamoran — Pulseras (modelo)</t>
+          <t>Piezas que enamoran — Pendientes — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="F14" s="22" t="inlineStr">
@@ -1185,12 +1194,12 @@
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
+          <t>Se muestra al pasar el ratón sobre la foto de Pendientes, sin hacer clic. Modelo llevando los pendientes, primer plano de rostro y oreja.</t>
         </is>
       </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
-          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
+          <t>Close-up of a woman's face wearing elegant gold earrings, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
       <c r="I14" s="25" t="inlineStr">
@@ -1210,7 +1219,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>home-destacado-1.jpg</t>
+          <t>home-slider-collares.jpg</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -1225,23 +1234,23 @@
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 1</t>
+          <t>Piezas que enamoran — Collares (estudio)</t>
         </is>
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad izquierda de la 2ª fila del slider a pantalla completa. Collares en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Fine gold necklaces and chains arranged on a neutral studio background, luxury jewelry product photography, soft shadows, minimal elegant composition, 8K</t>
         </is>
       </c>
       <c r="I15" s="24" t="inlineStr">
@@ -1261,7 +1270,7 @@
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>home-destacado-2.jpg</t>
+          <t>home-slider-collares-modelo.jpg</t>
         </is>
       </c>
       <c r="C16" s="22" t="inlineStr">
@@ -1276,23 +1285,23 @@
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 2</t>
+          <t>Piezas que enamoran — Collares — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="F16" s="22" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Se muestra al pasar el ratón sobre la foto de Collares, sin hacer clic. Modelo llevando el collar, plano de escote y cuello.</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Elegant woman wearing a fine gold necklace, close-up of neckline and collarbone, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
       <c r="I16" s="25" t="inlineStr">
@@ -1312,7 +1321,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>home-destacado-3.jpg</t>
+          <t>home-slider-pulseras.jpg</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1327,23 +1336,23 @@
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 3</t>
+          <t>Piezas que enamoran — Pulseras (estudio)</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Mitad derecha de la 2ª fila del slider a pantalla completa. Pulseras en foto de estudio sobre fondo neutro.</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Elegant gold bracelets arranged on a neutral cream studio background, luxury jewelry product photography, soft shadows, minimal composition, high-end editorial style, 8K</t>
         </is>
       </c>
       <c r="I17" s="24" t="inlineStr">
@@ -1363,7 +1372,7 @@
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>home-destacado-4.jpg</t>
+          <t>home-slider-pulseras-modelo.jpg</t>
         </is>
       </c>
       <c r="C18" s="22" t="inlineStr">
@@ -1378,23 +1387,23 @@
       </c>
       <c r="E18" s="22" t="inlineStr">
         <is>
-          <t>Piezas destacadas — pieza 4</t>
+          <t>Piezas que enamoran — Pulseras — 2ª foto en hover (modelo)</t>
         </is>
       </c>
       <c r="F18" s="22" t="inlineStr">
         <is>
-          <t>800×1000 px
-≤200 KB</t>
+          <t>1200×1500 px
+≤400 KB</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+          <t>Se muestra al pasar el ratón sobre la foto de Pulseras, sin hacer clic. Modelo llevando pulseras, plano de muñeca y antebrazo en primer plano.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+          <t>Close-up of a woman's wrist and forearm wearing elegant gold bracelets, editorial luxury jewelry campaign photography, soft natural light, neutral skin tones, shallow depth of field, high-end fashion style, 8K</t>
         </is>
       </c>
       <c r="I18" s="25" t="inlineStr">
@@ -1414,38 +1423,38 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>proceso-boceto.jpg</t>
+          <t>home-destacado-1.jpg</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Raíz del proyecto</t>
+          <t>images/home</t>
         </is>
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
         <is>
-          <t>Paso 1 — Boceto</t>
+          <t>Piezas destacadas — pieza 1</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="H19" s="17" t="inlineStr">
         <is>
-          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
       <c r="I19" s="24" t="inlineStr">
@@ -1465,38 +1474,38 @@
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>proceso-materiales.jpg</t>
+          <t>home-destacado-2.jpg</t>
         </is>
       </c>
       <c r="C20" s="22" t="inlineStr">
         <is>
-          <t>Raíz del proyecto</t>
+          <t>images/home</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="E20" s="22" t="inlineStr">
         <is>
-          <t>Paso 2 — Materiales</t>
+          <t>Piezas destacadas — pieza 2</t>
         </is>
       </c>
       <c r="F20" s="22" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="G20" s="21" t="inlineStr">
         <is>
-          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="H20" s="21" t="inlineStr">
         <is>
-          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
       <c r="I20" s="25" t="inlineStr">
@@ -1516,38 +1525,38 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>proceso-artesania.jpg</t>
+          <t>home-destacado-3.jpg</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Raíz del proyecto</t>
+          <t>images/home</t>
         </is>
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
         <is>
-          <t>Paso 3 — Artesanía</t>
+          <t>Piezas destacadas — pieza 3</t>
         </is>
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>900×600 px
+          <t>800×1000 px
 ≤200 KB</t>
         </is>
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
         </is>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
-          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
         </is>
       </c>
       <c r="I21" s="24" t="inlineStr">
@@ -1567,53 +1576,257 @@
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>proceso-entrega.jpg</t>
+          <t>home-destacado-4.jpg</t>
         </is>
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
+          <t>images/home</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>Piezas destacadas — pieza 4</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>800×1000 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="inlineStr">
+        <is>
+          <t>Pieza a definir. Foto de producto en estudio, fondo neutro, formato vertical, tira de 4 piezas bajo el slider.</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>Elegant gold jewelry piece on a neutral studio background, luxury product photography, soft shadows, vertical composition, minimal editorial style, 8K</t>
+        </is>
+      </c>
+      <c r="I22" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J22" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="70" customHeight="1" s="11">
+      <c r="A23" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>proceso-boceto.jpg</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
           <t>Raíz del proyecto</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>Atelier</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
-        <is>
-          <t>Paso 4 — Entrega</t>
-        </is>
-      </c>
-      <c r="F22" s="22" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Paso 1 — Boceto</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
         <is>
           <t>900×600 px
 ≤200 KB</t>
         </is>
       </c>
-      <c r="G22" s="21" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>Mano de diseñador dibujando boceto de joya sobre papel. Lápices, regla, mesa de diseño.</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>Jewelry designer hand sketching ring design on paper with pencils and ruler on wooden desk, warm light, artisan workshop, shallow depth of field, elegant craftsmanship photography, 8K</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J23" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="70" customHeight="1" s="11">
+      <c r="A24" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>proceso-materiales.jpg</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Paso 2 — Materiales</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="G24" s="21" t="inlineStr">
+        <is>
+          <t>Selección de metales preciosos y gemas en bruto sobre superficie neutra. Oro, plata, piedras.</t>
+        </is>
+      </c>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>Selection of precious metals gold and silver sheets, rough diamonds and colored gemstones on white marble, luxury jewelry materials flat lay, top view, elegant minimal photography, 8K</t>
+        </is>
+      </c>
+      <c r="I24" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J24" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="70" customHeight="1" s="11">
+      <c r="A25" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>proceso-artesania.jpg</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Paso 3 — Artesanía</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>Joyero trabajando con herramientas: soldando, puliendo o engastando una gema. Plano detalle de manos.</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>Expert goldsmith hands setting a diamond in a gold ring with precision tools in a jewelry workshop, focused macro photography, warm workshop lighting, artisan craftsmanship, 8K</t>
+        </is>
+      </c>
+      <c r="I25" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J25" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="70" customHeight="1" s="11">
+      <c r="A26" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>proceso-entrega.jpg</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>Raíz del proyecto</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>Paso 4 — Entrega</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>900×600 px
+≤200 KB</t>
+        </is>
+      </c>
+      <c r="G26" s="21" t="inlineStr">
         <is>
           <t>Joya terminada en estuche o caja de regalo de lujo. Momento de entrega o presentación.</t>
         </is>
       </c>
-      <c r="H22" s="21" t="inlineStr">
+      <c r="H26" s="21" t="inlineStr">
         <is>
           <t>Finished luxury gold ring inside an elegant black velvet jewelry box with ribbon, gift presentation, soft studio lighting, luxury brand photography, clean minimal background, 8K</t>
         </is>
       </c>
-      <c r="I22" s="25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J22" s="25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="I26" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J26" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>⚠️  Recuerda actualizar el dominio en sitemap.xml y robots.txt cuando tengas el dominio definitivo · Tamaños en px · Peso máximo recomendado por imagen · "¿La has hecho?": marca Sí cuando tengas la foto lista · "Subida a la web": lo actualizo yo automáticamente cuando detecto el archivo subido en la carpeta correspondiente · "Carpeta destino": dónde va cada archivo dentro del proyecto (raíz, o dentro de la carpeta images/home)</t>
         </is>
@@ -1621,14 +1834,11 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A28:J28"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation sqref="H5:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Sí"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I5:I22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="1">
+    <dataValidation sqref="I5:I26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Sí"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Comprimir home-destacado-1.jpg y marcar piezas destacadas como subidas
home-destacado-1.jpg pesaba 388 KB (2305×4096 px), por encima del
límite de 200 KB del checklist; se comprime a 64 KB sin pérdida de
calidad visible. Se marca "Subida a la web" = Sí para las 4 fotos de
estudio de piezas destacadas (quedan pendientes las 4 versiones
"modelo").

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -1451,9 +1451,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J19" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="J19" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1553,9 +1553,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J21" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1655,9 +1655,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J23" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="J23" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1757,9 +1757,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J25" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Comprimir home-destacado-1.jpg y marcar piezas destacadas como subidas (#16)
home-destacado-1.jpg pesaba 388 KB (2305×4096 px), por encima del
límite de 200 KB del checklist; se comprime a 64 KB sin pérdida de
calidad visible. Se marca "Subida a la web" = Sí para las 4 fotos de
estudio de piezas destacadas (quedan pendientes las 4 versiones
"modelo").


Claude-Session: https://claude.ai/code/session_012FBTtSqErTnTcS9bXg9i8X

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotos-web-checklist.xlsx
+++ b/fotos-web-checklist.xlsx
@@ -1451,9 +1451,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J19" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="J19" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1553,9 +1553,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J21" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1655,9 +1655,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J23" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="J23" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1757,9 +1757,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J25" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>